<commit_message>
Update inventory data 2026-09-18 09:16
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139ACDA5-A662-4A1A-99B8-45C38D56074B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457CE53E-4F83-4094-8285-3FE06574CC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="420" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1605" yWindow="1260" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="100">
   <si>
     <t>分類</t>
   </si>
@@ -362,17 +362,6 @@
   </si>
   <si>
     <t>8/17採購617卷，預計九月底完成</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/10採購120卷，預計9/17到貨，Sally預約80卷</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/10採購40卷，預計9/17到貨</t>
-  </si>
-  <si>
-    <t>9/10採購40卷，預計9/17到貨</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -1293,6 +1282,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52853FC6-D5F2-C342-BFD8-83BB6438EE86}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1631,7 +1674,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -1667,9 +1710,7 @@
       <c r="Q3" s="13">
         <v>40</v>
       </c>
-      <c r="R3" s="11" t="s">
-        <v>96</v>
-      </c>
+      <c r="R3" s="11"/>
       <c r="S3" s="10">
         <v>900</v>
       </c>
@@ -1780,9 +1821,7 @@
       <c r="O6" s="13"/>
       <c r="P6" s="13"/>
       <c r="Q6" s="13"/>
-      <c r="R6" s="11" t="s">
-        <v>98</v>
-      </c>
+      <c r="R6" s="11"/>
       <c r="S6" s="10">
         <v>960</v>
       </c>
@@ -1897,9 +1936,7 @@
       <c r="O9" s="13"/>
       <c r="P9" s="13"/>
       <c r="Q9" s="13"/>
-      <c r="R9" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="R9" s="8"/>
       <c r="S9" s="10">
         <v>960</v>
       </c>
@@ -1936,9 +1973,7 @@
       <c r="O10" s="13"/>
       <c r="P10" s="13"/>
       <c r="Q10" s="13"/>
-      <c r="R10" s="8" t="s">
-        <v>97</v>
-      </c>
+      <c r="R10" s="8"/>
       <c r="S10" s="10">
         <v>1200</v>
       </c>
@@ -2054,7 +2089,7 @@
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
       <c r="R13" s="11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="S13" s="10">
         <v>950</v>
@@ -2093,7 +2128,7 @@
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S14" s="10">
         <v>600</v>
@@ -2132,7 +2167,7 @@
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
       <c r="R15" s="11" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="S15" s="10">
         <v>600</v>
@@ -2171,7 +2206,7 @@
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
       <c r="R16" s="11" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="S16" s="10">
         <v>1400</v>

</xml_diff>

<commit_message>
Update inventory data 2026-09-22 14:02
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457CE53E-4F83-4094-8285-3FE06574CC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7927DC3-1E4F-44AB-A8F7-DFA34AB4D9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1605" yWindow="1260" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -361,23 +361,23 @@
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
   </si>
   <si>
-    <t>8/17採購617卷，預計九月底完成</t>
+    <t>9/10採購124卷，10/1或10/8送</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購411卷，交期未知</t>
+    <t>8/17採購617卷，10/1或10/8送</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購206卷，交期未知</t>
+    <t>9/10採購411卷，10/1送</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購124卷，交期未知</t>
+    <t>9/10採購206卷，10/1送</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/11採購103卷，交期未知</t>
+    <t>9/11採購103卷，10/1送</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1336,6 +1336,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E02868D-15F4-6DBD-EE80-EC2EFF70931E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2015,7 +2069,7 @@
         <v>120</v>
       </c>
       <c r="R11" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S11" s="10">
         <v>990</v>
@@ -2089,7 +2143,7 @@
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
       <c r="R13" s="11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="S13" s="10">
         <v>950</v>
@@ -2128,7 +2182,7 @@
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S14" s="10">
         <v>600</v>
@@ -2167,7 +2221,7 @@
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
       <c r="R15" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="S15" s="10">
         <v>600</v>

</xml_diff>

<commit_message>
Update inventory data 2026-09-22 15:15
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7927DC3-1E4F-44AB-A8F7-DFA34AB4D9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5212BA5-D9A1-49F5-B5CB-327E7BCD8B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1605" yWindow="1260" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="101">
   <si>
     <t>分類</t>
   </si>
@@ -361,23 +361,27 @@
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
   </si>
   <si>
-    <t>9/10採購124卷，10/1或10/8送</t>
+    <t>9/11採購103卷，10/1送10/2: 中40R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>8/17採購617卷，10/1或10/8送</t>
+    <t>9/10採購124卷，10/1: 南</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購411卷，10/1送</t>
+    <t>8/17採購617卷，10/1: 南xR；10/2: 北120R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購206卷，10/1送</t>
+    <t>9/10採購206卷，10/1: 南xR；10/2: 高60R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/11採購103卷，10/1送</t>
+    <t>9/10採購411卷，10/1: 南xR；10/2: 北120R、中120R、 高60R</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/11採購103卷，10/1: 南xR；10/2: 中40R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1390,6 +1394,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CCF0A1C-198E-B21B-F4C7-A33AFFFEF73E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2069,7 +2127,7 @@
         <v>120</v>
       </c>
       <c r="R11" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S11" s="10">
         <v>990</v>
@@ -2143,7 +2201,7 @@
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
       <c r="R13" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S13" s="10">
         <v>950</v>
@@ -2182,7 +2240,7 @@
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="S14" s="10">
         <v>600</v>
@@ -2260,7 +2318,7 @@
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
       <c r="R16" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S16" s="10">
         <v>1400</v>

</xml_diff>

<commit_message>
Update inventory data 2026-09-30 11:41
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5212BA5-D9A1-49F5-B5CB-327E7BCD8B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C85ACDD-2FE8-476E-A25C-61C92EF05D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1605" yWindow="1260" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1215" yWindow="1050" windowWidth="20640" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="100">
   <si>
     <t>分類</t>
   </si>
@@ -361,27 +361,23 @@
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
   </si>
   <si>
-    <t>9/11採購103卷，10/1送10/2: 中40R</t>
+    <t>8/17採購617卷，10/1: 南490R；10/2: 北120R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購124卷，10/1: 南</t>
+    <t>9/10採購124卷，10/1: 南120R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>8/17採購617卷，10/1: 南xR；10/2: 北120R</t>
+    <t>9/10採購206卷，10/1: 南144R；10/2: 高60R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購206卷，10/1: 南xR；10/2: 高60R</t>
+    <t>9/10採購411卷，10/1: 南108R；10/2: 北120R、中120R、 高60R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>9/10採購411卷，10/1: 南xR；10/2: 北120R、中120R、 高60R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/11採購103卷，10/1: 南xR；10/2: 中40R</t>
+    <t>9/11採購103卷，10/1: 南61R；10/2: 中40R</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1448,6 +1444,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70BEFB36-C8DF-4191-67AE-F8A020DAC98E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2127,7 +2177,7 @@
         <v>120</v>
       </c>
       <c r="R11" s="11" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="S11" s="10">
         <v>990</v>
@@ -2240,7 +2290,7 @@
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="S14" s="10">
         <v>600</v>
@@ -2279,7 +2329,7 @@
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
       <c r="R15" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="S15" s="10">
         <v>600</v>
@@ -2318,7 +2368,7 @@
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
       <c r="R16" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="S16" s="10">
         <v>1400</v>

</xml_diff>

<commit_message>
Update inventory data 2026-10-05 09:14
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C85ACDD-2FE8-476E-A25C-61C92EF05D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F4B855-ADBB-42A7-AF90-B819207B6F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1215" yWindow="1050" windowWidth="20640" windowHeight="14460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1245" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="95">
   <si>
     <t>分類</t>
   </si>
@@ -359,26 +359,6 @@
   </si>
   <si>
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
-  </si>
-  <si>
-    <t>8/17採購617卷，10/1: 南490R；10/2: 北120R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/10採購124卷，10/1: 南120R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/10採購206卷，10/1: 南144R；10/2: 高60R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/10採購411卷，10/1: 南108R；10/2: 北120R、中120R、 高60R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>9/11採購103卷，10/1: 南61R；10/2: 中40R</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1498,6 +1478,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F80E53D0-31AB-2AF4-AA40-6B4FEBCE91B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2176,9 +2210,7 @@
       <c r="Q11" s="13">
         <v>120</v>
       </c>
-      <c r="R11" s="11" t="s">
-        <v>95</v>
-      </c>
+      <c r="R11" s="11"/>
       <c r="S11" s="10">
         <v>990</v>
       </c>
@@ -2250,9 +2282,7 @@
       <c r="O13" s="13"/>
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
-      <c r="R13" s="11" t="s">
-        <v>96</v>
-      </c>
+      <c r="R13" s="11"/>
       <c r="S13" s="10">
         <v>950</v>
       </c>
@@ -2289,9 +2319,7 @@
       <c r="O14" s="13"/>
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
-      <c r="R14" s="11" t="s">
-        <v>98</v>
-      </c>
+      <c r="R14" s="11"/>
       <c r="S14" s="10">
         <v>600</v>
       </c>
@@ -2328,9 +2356,7 @@
       <c r="O15" s="13"/>
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
-      <c r="R15" s="11" t="s">
-        <v>97</v>
-      </c>
+      <c r="R15" s="11"/>
       <c r="S15" s="10">
         <v>600</v>
       </c>
@@ -2367,9 +2393,7 @@
       <c r="O16" s="13"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="11" t="s">
-        <v>99</v>
-      </c>
+      <c r="R16" s="11"/>
       <c r="S16" s="10">
         <v>1400</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-10-08 09:14
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F4B855-ADBB-42A7-AF90-B819207B6F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC098DA3-0237-4FAB-A445-39BD40CF0452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="1245" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1532,6 +1532,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B7434F2-2DC3-19D5-5CD8-436871A65C88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1847,12 +1901,8 @@
       </c>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
-      <c r="H2" s="13">
-        <v>100</v>
-      </c>
-      <c r="I2" s="13">
-        <v>60</v>
-      </c>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
@@ -1900,12 +1950,8 @@
       <c r="M3" s="13"/>
       <c r="N3" s="13"/>
       <c r="O3" s="13"/>
-      <c r="P3" s="13">
-        <v>60</v>
-      </c>
-      <c r="Q3" s="13">
-        <v>40</v>
-      </c>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
       <c r="R3" s="11"/>
       <c r="S3" s="10">
         <v>900</v>
@@ -1927,12 +1973,8 @@
       <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="13">
-        <v>100</v>
-      </c>
-      <c r="G4" s="13">
-        <v>60</v>
-      </c>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
       <c r="H4" s="13"/>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
@@ -1941,8 +1983,12 @@
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
+      <c r="P4" s="13">
+        <v>100</v>
+      </c>
+      <c r="Q4" s="13">
+        <v>60</v>
+      </c>
       <c r="R4" s="8"/>
       <c r="S4" s="10">
         <v>540</v>
@@ -1968,18 +2014,18 @@
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
       <c r="I5" s="13"/>
-      <c r="J5" s="13">
-        <v>100</v>
-      </c>
-      <c r="K5" s="13">
-        <v>60</v>
-      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
       <c r="N5" s="13"/>
       <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
+      <c r="P5" s="13">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="13">
+        <v>100</v>
+      </c>
       <c r="R5" s="11"/>
       <c r="S5" s="10">
         <v>600</v>
@@ -2079,12 +2125,8 @@
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
-      <c r="J8" s="13">
-        <v>50</v>
-      </c>
-      <c r="K8" s="13">
-        <v>30</v>
-      </c>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -2273,9 +2315,7 @@
       <c r="H13" s="13"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="13">
-        <v>10</v>
-      </c>
+      <c r="K13" s="13"/>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2317,8 +2357,12 @@
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
       <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
+      <c r="P14" s="13">
+        <v>150</v>
+      </c>
+      <c r="Q14" s="13">
+        <v>80</v>
+      </c>
       <c r="R14" s="11"/>
       <c r="S14" s="10">
         <v>600</v>
@@ -2354,8 +2398,12 @@
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
+      <c r="P15" s="13">
+        <v>150</v>
+      </c>
+      <c r="Q15" s="13">
+        <v>50</v>
+      </c>
       <c r="R15" s="11"/>
       <c r="S15" s="10">
         <v>600</v>
@@ -2533,12 +2581,8 @@
       <c r="M20" s="13"/>
       <c r="N20" s="13"/>
       <c r="O20" s="13"/>
-      <c r="P20" s="13">
-        <v>20</v>
-      </c>
-      <c r="Q20" s="13">
-        <v>8</v>
-      </c>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
       <c r="R20" s="8"/>
       <c r="S20" s="10"/>
     </row>
@@ -2568,9 +2612,7 @@
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
       <c r="O21" s="13"/>
-      <c r="P21" s="13">
-        <v>20</v>
-      </c>
+      <c r="P21" s="13"/>
       <c r="Q21" s="13"/>
       <c r="R21" s="8"/>
       <c r="S21" s="10"/>
@@ -2727,12 +2769,8 @@
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
       <c r="I26" s="13"/>
-      <c r="J26" s="13">
-        <v>60</v>
-      </c>
-      <c r="K26" s="13">
-        <v>40</v>
-      </c>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
       <c r="L26" s="13"/>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -2863,12 +2901,8 @@
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
       <c r="I30" s="13"/>
-      <c r="J30" s="13">
-        <v>60</v>
-      </c>
-      <c r="K30" s="13">
-        <v>40</v>
-      </c>
+      <c r="J30" s="13"/>
+      <c r="K30" s="13"/>
       <c r="L30" s="13"/>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -2900,12 +2934,8 @@
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
       <c r="I31" s="13"/>
-      <c r="J31" s="13">
-        <v>60</v>
-      </c>
-      <c r="K31" s="13">
-        <v>40</v>
-      </c>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
       <c r="L31" s="13"/>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>

</xml_diff>

<commit_message>
Update inventory data 2026-10-14 11:32
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC098DA3-0237-4FAB-A445-39BD40CF0452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE27A8C-DC39-4473-B28E-32D728ADB2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1245" windowWidth="20640" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1245" windowWidth="18765" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -1586,6 +1586,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DB24B85-D7DE-7DC5-A3AD-97BDC7D224DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1917,7 +1971,7 @@
       </c>
       <c r="R2" s="11"/>
       <c r="S2" s="10">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1954,7 +2008,7 @@
       <c r="Q3" s="13"/>
       <c r="R3" s="11"/>
       <c r="S3" s="10">
-        <v>900</v>
+        <v>850</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -1991,7 +2045,7 @@
       </c>
       <c r="R4" s="8"/>
       <c r="S4" s="10">
-        <v>540</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -2028,7 +2082,7 @@
       </c>
       <c r="R5" s="11"/>
       <c r="S5" s="10">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -2065,7 +2119,7 @@
       <c r="Q6" s="13"/>
       <c r="R6" s="11"/>
       <c r="S6" s="10">
-        <v>960</v>
+        <v>900</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -2102,7 +2156,7 @@
       <c r="Q7" s="13"/>
       <c r="R7" s="8"/>
       <c r="S7" s="10">
-        <v>1200</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -2139,7 +2193,7 @@
       </c>
       <c r="R8" s="8"/>
       <c r="S8" s="10">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -2176,7 +2230,7 @@
       <c r="Q9" s="13"/>
       <c r="R9" s="8"/>
       <c r="S9" s="10">
-        <v>960</v>
+        <v>900</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2213,7 +2267,7 @@
       <c r="Q10" s="13"/>
       <c r="R10" s="8"/>
       <c r="S10" s="10">
-        <v>1200</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2254,7 +2308,7 @@
       </c>
       <c r="R11" s="11"/>
       <c r="S11" s="10">
-        <v>990</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2348,10 +2402,10 @@
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K14" s="13">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
@@ -2365,7 +2419,7 @@
       </c>
       <c r="R14" s="11"/>
       <c r="S14" s="10">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2406,7 +2460,7 @@
       </c>
       <c r="R15" s="11"/>
       <c r="S15" s="10">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2443,7 +2497,7 @@
       <c r="Q16" s="13"/>
       <c r="R16" s="11"/>
       <c r="S16" s="10">
-        <v>1400</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2480,7 +2534,7 @@
       </c>
       <c r="R17" s="8"/>
       <c r="S17" s="10">
-        <v>1200</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2517,7 +2571,7 @@
       </c>
       <c r="R18" s="11"/>
       <c r="S18" s="10">
-        <v>1200</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2553,7 +2607,9 @@
       <c r="P19" s="13"/>
       <c r="Q19" s="13"/>
       <c r="R19" s="8"/>
-      <c r="S19" s="10"/>
+      <c r="S19" s="10">
+        <v>1600</v>
+      </c>
     </row>
     <row r="20" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -2712,7 +2768,9 @@
       <c r="P24" s="13"/>
       <c r="Q24" s="13"/>
       <c r="R24" s="8"/>
-      <c r="S24" s="10"/>
+      <c r="S24" s="10">
+        <v>900</v>
+      </c>
     </row>
     <row r="25" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">

</xml_diff>

<commit_message>
Update inventory data 2026-10-20 15:51
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE27A8C-DC39-4473-B28E-32D728ADB2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2279192-E038-46F1-A78D-6C81475E0097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1245" windowWidth="18765" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3690" yWindow="1665" windowWidth="18765" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -1640,6 +1640,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77CE0BD8-4D88-AA69-0464-C3365D5000A2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2567,7 +2621,7 @@
         <v>100</v>
       </c>
       <c r="Q18" s="13">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="R18" s="11"/>
       <c r="S18" s="10">

</xml_diff>

<commit_message>
Update inventory data 2026-10-28 09:16
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2279192-E038-46F1-A78D-6C81475E0097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB994871-F93E-4918-BE99-4B98D53E52C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3690" yWindow="1665" windowWidth="18765" windowHeight="13245" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>分類</t>
   </si>
@@ -359,6 +359,14 @@
   </si>
   <si>
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
+  </si>
+  <si>
+    <t>10/27採購96卷，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>10/27採購51卷，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1694,6 +1702,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BCC77B2-0043-4A16-F6DC-7287F55E9C07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2549,7 +2611,9 @@
       <c r="O16" s="13"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="11"/>
+      <c r="R16" s="11" t="s">
+        <v>96</v>
+      </c>
       <c r="S16" s="10">
         <v>1500</v>
       </c>
@@ -2623,7 +2687,9 @@
       <c r="Q18" s="13">
         <v>60</v>
       </c>
-      <c r="R18" s="11"/>
+      <c r="R18" s="11" t="s">
+        <v>95</v>
+      </c>
       <c r="S18" s="10">
         <v>1300</v>
       </c>

</xml_diff>